<commit_message>
Address BMC Women's Health review scope fixes
</commit_message>
<xml_diff>
--- a/manuscript_submission_snapshot/additional_files/additional_file_1_harmonization_and_cohort_construction.xlsx
+++ b/manuscript_submission_snapshot/additional_files/additional_file_1_harmonization_and_cohort_construction.xlsx
@@ -7,11 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="item_crosswalk" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cohort_tier_lock" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="harmonization_risk_matrix" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="baseline_covariates" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sheet_index" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="item_crosswalk" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cohort_tier_lock" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="harmonization_risk_matrix" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="baseline_covariates" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="age_distribution" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -33,12 +35,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -53,9 +60,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -421,6 +429,108 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>sheet_name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>README</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Workbook overview.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>item_crosswalk</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Item-level cohort-domain harmonization crosswalk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>cohort_tier_lock</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Locked evidence-tier and analysis-role definitions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>harmonization_risk_matrix</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Cohort-by-domain measurement risk matrix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>baseline_covariates</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Baseline clinical, design and covariate availability metadata.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>age_distribution</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Women aged 50 years or older split into 50-64 and 65+ strata by cohort.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -490,7 +600,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
@@ -598,7 +707,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12103,7 +12212,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12831,7 +12940,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14423,7 +14532,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14822,4 +14931,347 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="27" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>cohort</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>source_age_nonmissing_n</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>source_age_50_64_n</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>source_age_50_64_pct</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>source_age_ge65_n</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>source_age_ge65_pct</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>complete_age_nonmissing_n</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>complete_age_50_64_n</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>complete_age_50_64_pct</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>complete_age_ge65_n</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>complete_age_ge65_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CHARLS</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>6878</v>
+      </c>
+      <c r="C2" t="n">
+        <v>4536</v>
+      </c>
+      <c r="D2" t="n">
+        <v>65.90000000000001</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2342</v>
+      </c>
+      <c r="F2" t="n">
+        <v>34.1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>6019</v>
+      </c>
+      <c r="H2" t="n">
+        <v>4081</v>
+      </c>
+      <c r="I2" t="n">
+        <v>67.8</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1938</v>
+      </c>
+      <c r="K2" t="n">
+        <v>32.2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ELSA</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>6292</v>
+      </c>
+      <c r="C3" t="n">
+        <v>3210</v>
+      </c>
+      <c r="D3" t="n">
+        <v>51</v>
+      </c>
+      <c r="E3" t="n">
+        <v>3082</v>
+      </c>
+      <c r="F3" t="n">
+        <v>49</v>
+      </c>
+      <c r="G3" t="n">
+        <v>6104</v>
+      </c>
+      <c r="H3" t="n">
+        <v>3151</v>
+      </c>
+      <c r="I3" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="J3" t="n">
+        <v>2953</v>
+      </c>
+      <c r="K3" t="n">
+        <v>48.4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HRS</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>11005</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4797</v>
+      </c>
+      <c r="D4" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="E4" t="n">
+        <v>6208</v>
+      </c>
+      <c r="F4" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="G4" t="n">
+        <v>10202</v>
+      </c>
+      <c r="H4" t="n">
+        <v>4636</v>
+      </c>
+      <c r="I4" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="J4" t="n">
+        <v>5566</v>
+      </c>
+      <c r="K4" t="n">
+        <v>54.6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>KLoSA</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4344</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D5" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2328</v>
+      </c>
+      <c r="F5" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4081</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1923</v>
+      </c>
+      <c r="I5" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="J5" t="n">
+        <v>2158</v>
+      </c>
+      <c r="K5" t="n">
+        <v>52.9</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>LASI</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>28165</v>
+      </c>
+      <c r="C6" t="n">
+        <v>17158</v>
+      </c>
+      <c r="D6" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="E6" t="n">
+        <v>11007</v>
+      </c>
+      <c r="F6" t="n">
+        <v>39.1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>27433</v>
+      </c>
+      <c r="H6" t="n">
+        <v>16865</v>
+      </c>
+      <c r="I6" t="n">
+        <v>61.5</v>
+      </c>
+      <c r="J6" t="n">
+        <v>10568</v>
+      </c>
+      <c r="K6" t="n">
+        <v>38.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>MHAS</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>7440</v>
+      </c>
+      <c r="C7" t="n">
+        <v>4640</v>
+      </c>
+      <c r="D7" t="n">
+        <v>62.4</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2800</v>
+      </c>
+      <c r="F7" t="n">
+        <v>37.6</v>
+      </c>
+      <c r="G7" t="n">
+        <v>6733</v>
+      </c>
+      <c r="H7" t="n">
+        <v>4293</v>
+      </c>
+      <c r="I7" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="J7" t="n">
+        <v>2440</v>
+      </c>
+      <c r="K7" t="n">
+        <v>36.2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SHARE</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>15814</v>
+      </c>
+      <c r="C8" t="n">
+        <v>8513</v>
+      </c>
+      <c r="D8" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="E8" t="n">
+        <v>7301</v>
+      </c>
+      <c r="F8" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>15721</v>
+      </c>
+      <c r="H8" t="n">
+        <v>8475</v>
+      </c>
+      <c r="I8" t="n">
+        <v>53.9</v>
+      </c>
+      <c r="J8" t="n">
+        <v>7246</v>
+      </c>
+      <c r="K8" t="n">
+        <v>46.1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>